<commit_message>
Expand UT/ST summary to 28 defects
Added 11 previously missed defects from commit history:
- UT-002: LengthHW wrong return type (uint→int)
- UT-004: Short/UShort missing in constant expression
- UT-007: CoopVec wrong extension name
- UT-009: Optional use operand crash (word_count=5)
- UT-011: CoopMatHW opcode 65xx→66xx
- UT-012: cp-async/shuffle opcode 6466→6613
- UT-016: Extension naming inconsistency (3 names→1)
- ST-003: Missing non-GLSL backend rejection
- ST-004: Missing Vulkan GLSL test coverage
- ST-005: Missing MSL/HLSL rejection test coverage
- ST-006: Missing glslang roundtrip validation

24 closed, 4 open. Header frozen, auto-filter, summary stats.
</commit_message>
<xml_diff>
--- a/doc/hw-ut-st-summary.xlsx
+++ b/doc/hw-ut-st-summary.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="研发自测UT-ST缺陷总结表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'研发自测UT-ST缺陷总结表'!$A$1:$L$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'研发自测UT-ST缺陷总结表'!$A$1:$L$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,6 +39,10 @@
       <b val="1"/>
       <color rgb="00FF0000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -91,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -111,6 +115,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,16 +482,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -628,17 +634,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>coopmatHW&lt;float,16,16&gt;(100.0f)作为立即数传给coopMatStore时抛"Invalid constant expression basetype"，CoopMatHW未在constant_expression中处理</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>OpCooperativeMatrixLengthHW返回类型为uint，应为int（有符号32位整数）</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>新增类型未覆盖所有类型分发分支，constant_expression遗漏CoopMatHW case</t>
+          <t>返回类型与设计规范不一致，设计规范要求OpTypeInt(32-bit signed)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -648,7 +654,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>构造coopmatHW常量值传入Store操作</t>
+          <t>LengthHW结果用于有符号运算时类型不匹配</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -658,12 +664,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
@@ -688,7 +694,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>coopMatReduceHW返回coopmatHW&lt;T,M,N&gt;，但实现用void out-param模式，未生成返回值赋值</t>
+          <t>coopmatHW&lt;float,16,16&gt;(100.0f)作为立即数传给coopMatStore时抛"Invalid constant expression basetype"，CoopMatHW未在constant_expression中处理</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -698,7 +704,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>函数签名理解错误：ReduceHW有返回值而非void out-param，与MulAddHW（void out-param）混淆</t>
+          <t>新增类型未覆盖所有类型分发分支，constant_expression遗漏CoopMatHW case</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -708,7 +714,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>编译含ReduceHW的shader后输出缺少返回值</t>
+          <t>构造coopmatHW常量值传入Store操作</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -718,12 +724,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
@@ -748,7 +754,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>coopmatMulHW（无C矩阵）只检测OpUndef，漏检OpConstantNull，传入OpConstantNull时错误生成coopMatMulAddHW</t>
+          <t>CoopMatHW常量表达式不支持Short/UShort组件类型，仅处理Float/Half/Int/UInt</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -758,7 +764,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>NULL检测不完整：只处理OpUndef，遗漏OpConstantNull</t>
+          <t>constant_expression中CoopMatHW分支遗漏Short/UShort case</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -768,7 +774,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>使用OpConstantNull表示无C矩阵</t>
+          <t>使用int16_t/uint16_t组件类型的coopmatHW常量</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -778,12 +784,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
@@ -808,7 +814,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>CoopMatHW间OpBitcast（如float16→int16）错误使用构造函数，应使用float16BitsToInt16等bitcast函数</t>
+          <t>coopMatReduceHW返回coopmatHW&lt;T,M,N&gt;，但实现用void out-param模式，未生成返回值赋值</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -818,7 +824,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>OpBitcast分支未区分CoopMatHW间转换，直接走构造函数路径</t>
+          <t>函数签名理解错误：ReduceHW有返回值而非void out-param，与MulAddHW混淆</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -828,7 +834,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>CoopMatHW类型间执行OpBitcast</t>
+          <t>编译含ReduceHW的shader后输出缺少返回值</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -838,12 +844,12 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
@@ -868,17 +874,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>CoopVecHW未在access chain中处理，vec[i]索引无法生成，OpCompositeExtract/Insert崩溃</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>coopmatMulHW（无C矩阵）只检测OpUndef，漏检OpConstantNull，传入OpConstantNull时错误生成coopMatMulAddHW</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>新增CoopVecHW类型时未同步更新access_chain_internal和flattened_access_chain_offset</t>
+          <t>NULL检测不完整：只处理OpUndef，遗漏OpConstantNull</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -888,7 +894,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>对CoopVecHW执行组件索引访问</t>
+          <t>使用OpConstantNull表示无C矩阵</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -898,12 +904,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
@@ -911,7 +917,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>UT-单元功能验证</t>
+          <t>UT-边界值验证</t>
         </is>
       </c>
     </row>
@@ -928,7 +934,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>同宽整数CoopMatHW/CoopVecHW间bitcast（如int16→uint16）错误使用标量bitcast函数而非类型构造函数</t>
+          <t>CoopVecHW扩展名用了GL_HW_neural_shader，与CoopMatHW的GL_HW_neural_matrix不一致</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -938,7 +944,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>bitcast分支未区分同宽整数转换场景，应走构造函数而非bitcast函数</t>
+          <t>不同HW类型使用了不同的GLSL扩展名，未统一</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -948,7 +954,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>同宽整数CoopMatHW间执行OpBitcast</t>
+          <t>编译含CoopVecHW的shader时扩展声明不匹配</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -958,12 +964,12 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="K8" s="2" t="n">
@@ -988,7 +994,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>矩阵维度用get_constant().scalar()读取，不支持spec constant维度，spec constant场景崩溃</t>
+          <t>CoopMatHW间OpBitcast（如float16→int16）错误使用构造函数，应使用float16BitsToInt16等bitcast函数</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -998,7 +1004,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>使用get_constant而非evaluate_constant_u32，前者仅支持OpConstant不支持OpSpecConstant</t>
+          <t>OpBitcast分支未区分CoopMatHW间转换，直接走构造函数路径</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1008,7 +1014,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>使用spec constant指定矩阵行列数</t>
+          <t>CoopMatHW类型间执行OpBitcast</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1018,12 +1024,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
@@ -1031,7 +1037,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>UT-边界值验证</t>
+          <t>UT-单元功能验证</t>
         </is>
       </c>
     </row>
@@ -1048,17 +1054,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>reg_control未声明GL_HW_neural_shader扩展，且与flatten/branch hint共存时生成两个独立attribute而非合并形式</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>OpTypeCooperativeMatrixHW解析器假定use操作数总是存在（word_count=6），部分glslang生成的SPV省略use（word_count=5）导致越界</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>未处理attribute合并逻辑，glslang要求合并为单个[[flatten,reg_control]]</t>
+          <t>未处理可选操作数，直接访问ops[4]无长度检查</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1068,7 +1074,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>reg_control与flatten/branch hint同时使用</t>
+          <t>glslang生成的SPV省略CooperativeMatrixUse操作数</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1078,12 +1084,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="K10" s="2" t="n">
@@ -1091,7 +1097,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>UT-单元功能验证</t>
+          <t>UT-边界值验证</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1114,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>layout操作数用get&lt;SPIRConstant&gt;强转，当layout为三目运算符（OpSelect/OpSpecConstantOp）时抛bad_cast异常</t>
+          <t>CoopVecHW未在access chain中处理，vec[i]索引无法生成，OpCompositeExtract/Insert崩溃</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1118,7 +1124,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>未考虑layout操作数可能为非SPIRConstant类型，直接强转导致bad_cast</t>
+          <t>新增CoopVecHW类型时未同步更新access_chain_internal和flattened_access_chain_offset</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1128,7 +1134,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>使用三目运算符选择layout（cond?RowMajor:ColumnMajor）</t>
+          <t>对CoopVecHW执行组件索引访问</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1138,12 +1144,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="K11" s="2" t="n">
@@ -1151,14 +1157,14 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>UT-边界值验证</t>
+          <t>UT-单元功能验证</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ST-001</t>
+          <t>UT-011</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1168,17 +1174,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>函数名大小写错误：coopmatMulAddHW/coopmatMulHW应为coopMatMulAddHW/coopMatMulHW</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>CoopMatHW指令opcode编号错误：初始用65xx（6500-6505），设计规范要求66xx（6601-6606）</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>GLSL intrinsic函数名camelCase写成全小写，与扩展规范不一致</t>
+          <t>opcode编号与设计规范不一致，导致SPIR-V二进制无法被正确解析</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1188,7 +1194,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>回归测试比对参考文件发现输出函数名不匹配</t>
+          <t>使用正确opcode编号的SPV文件测试</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1198,12 +1204,12 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="K12" s="2" t="n">
@@ -1211,14 +1217,14 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>ST-回归测试</t>
+          <t>UT-接口验证</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>ST-002</t>
+          <t>UT-012</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1228,7 +1234,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>OpCooperativeMatrixStoreHW操作数顺序错误：代码按(Object,Pointer)读取，实际SPIR-V定义为(Pointer,Object)</t>
+          <t>cp-async/shuffle指令opcode编号错误：初始用6466-6480，设计规范要求6613-6621</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1238,7 +1244,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>SPIR-V指令操作数顺序与标准OpStore不一致，开发时按错误顺序解析，影响3处</t>
+          <t>opcode编号与设计规范不一致，与CoopMatHW的66xx范围不连续</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1248,7 +1254,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>回归测试59个用例后发现Store变量追踪异常</t>
+          <t>使用正确opcode编号的cp-async SPV文件测试</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1258,12 +1264,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
@@ -1271,14 +1277,14 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>ST-回归测试</t>
+          <t>UT-接口验证</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CR-001</t>
+          <t>UT-013</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1288,27 +1294,27 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>reject_hw_neural_extensions扩展检测用rfind("SPV_HW_",0)前缀匹配，过于宽泛，可能误拒未来其他SPV_HW_*扩展</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>同宽整数CoopMatHW/CoopVecHW间bitcast（如int16→uint16）错误使用标量bitcast函数而非类型构造函数</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>前缀匹配范围过大，应精确匹配SPV_HW_neural_shader</t>
+          <t>bitcast分支未区分同宽整数转换场景，应走构造函数而非bitcast函数</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>代码审查</t>
+          <t>开发自测</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>审查后端拒绝函数的扩展匹配逻辑</t>
+          <t>同宽整数CoopMatHW间执行OpBitcast</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1318,12 +1324,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="K14" s="2" t="n">
@@ -1331,14 +1337,14 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>代码审查-逻辑审查</t>
+          <t>UT-单元功能验证</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CR-002</t>
+          <t>UT-014</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1348,51 +1354,57 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>OpCooperativeMatrixLengthHW缺少length检查，直接访问ops[0~2]，若SPIR-V指令长度不足3会越界</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>中</t>
+          <t>矩阵维度用get_constant().scalar()读取，不支持spec constant维度，spec constant场景崩溃</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>遗漏bounds check，其他HW指令都有length保护</t>
+          <t>使用get_constant而非evaluate_constant_u32，前者仅支持OpConstant不支持OpSpecConstant</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>代码审查</t>
+          <t>开发自测</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>审查HW指令的length校验一致性</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>未关闭</t>
+          <t>使用spec constant指定矩阵行列数</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr"/>
-      <c r="K15" s="2" t="inlineStr"/>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>代码审查-安全性审查</t>
+          <t>UT-边界值验证</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CR-003</t>
+          <t>UT-015</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1402,51 +1414,57 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>OpCooperativeMatrixReduceHW的reduce_mask_id和combine_op_id用get&lt;SPIRConstant&gt;强转，与layout bug同一模式</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>高</t>
+          <t>reg_control未声明GL_HW_neural_shader扩展，且与flatten/branch hint共存时生成两个独立attribute而非合并形式</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>未参考layout修复模式同步修正ReduceHW的常量强转</t>
+          <t>未处理attribute合并逻辑，glslang要求合并为单个[[flatten,reg_control]]</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>代码审查</t>
+          <t>开发自测</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>审查ReduceHW实现发现与已修复的layout bug相同模式</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>未关闭</t>
+          <t>reg_control与flatten/branch hint同时使用</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr"/>
-      <c r="K16" s="2" t="inlineStr"/>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>代码审查-一致性审查</t>
+          <t>UT-单元功能验证</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CR-004</t>
+          <t>UT-016</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1456,103 +1474,782 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>OpCooperativeMatrixReduceHW的mask只判断==0否则当Column，op只判断0/1否则当Max，未校验范围，越界值静默走错枚举</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>低</t>
+          <t>CoopMatHW/CoopVecHW/TensorMap扩展名不统一：CoopMat用GL_HW_neural_matrix，CoopVec用GL_HW_cooperative_vector，应统一为GL_HW_neural_shader</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>缺少枚举值范围校验，越界值静默处理</t>
+          <t>多个HW类型使用了3个不同扩展名，未统一到单一扩展</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>代码审查</t>
+          <t>开发自测</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>审查ReduceHW的枚举值分发逻辑</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>未关闭</t>
+          <t>同时使用CoopMat和CoopVec的shader扩展声明冲突</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr"/>
-      <c r="K17" s="2" t="inlineStr"/>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>代码审查-逻辑审查</t>
+          <t>UT-单元功能验证</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>UT-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>layout操作数用get&lt;SPIRConstant&gt;强转，当layout为三目运算符（OpSelect/OpSpecConstantOp）时抛bad_cast异常</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>未考虑layout操作数可能为非SPIRConstant类型，直接强转导致bad_cast</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>开发自测</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>使用三目运算符选择layout（cond?RowMajor:ColumnMajor）</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>UT-边界值验证</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ST-001</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>函数名大小写错误：coopmatMulAddHW/coopmatMulHW应为coopMatMulAddHW/coopMatMulHW</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>GLSL intrinsic函数名camelCase写成全小写，与扩展规范不一致</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>开发自测</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>59个回归测试用例比对参考文件发现函数名不匹配</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>ST-回归测试</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ST-002</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>OpCooperativeMatrixStoreHW操作数顺序错误：代码按(Object,Pointer)读取，实际SPIR-V定义为(Pointer,Object)，影响3处（emit、interface tracking、scope analysis）</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>设计规范变更时操作数顺序理解错误，未遵循标准OpStore约定（Pointer在前Object在后）</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>开发自测</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>59个回归测试用例发现Store变量追踪异常</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>ST-回归测试</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ST-003</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>非GLSL后端（MSL/HLSL/CPP/Reflect）对HW扩展静默生成错误代码：HW指令经default分支落入基类CompilerGLSL::emit_instruction，将GLSL intrinsic写入MSL/HLSL输出</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>缺少后端拒绝机制，HW指令未在非GLSL后端入口处拦截</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>开发自测</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>用spirv-cross --msl转换HW shader发现输出含GLSL intrinsic</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>ST-兼容性测试</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ST-004</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Vulkan GLSL输出未覆盖：所有HW shader仅有OpenGL GLSL测试，缺少--vulkan-semantics(-V)输出验证</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>测试用例缺少.vk.标记，未触发Vulkan GLSL输出路径</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>开发自测</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>添加.vk.nocompat.变体后发现Vulkan GLSL输出与OpenGL有差异</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>ST-兼容性测试</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ST-005</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>MSL/HLSL后端拒绝测试未覆盖：虽有reject机制但无回归用例验证所有HW shader均被拒绝</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>测试基础设施缺少expected-error机制，无法验证拒绝行为</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>开发自测</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>添加MSL/HLSL拒绝测试段后发现130个shader全部正确拒绝</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>ST-兼容性测试</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ST-006</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>spirv-cross还原的GLSL代码未验证能否被glslang编译回去，存在输出语法错误的风险</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>测试流程缺少roundtrip验证步骤（spirv-cross输出→glslang编译）</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>开发自测</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>手动验证ternary layout输出的OpenGL和Vulkan GLSL均能编译</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>ST-回归测试</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>CR-001</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>reject_hw_neural_extensions扩展检测用rfind("SPV_HW_",0)前缀匹配，过于宽泛，可能误拒未来其他SPV_HW_*扩展</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>前缀匹配范围过大，应精确匹配SPV_HW_neural_shader</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>审查后端拒绝函数的扩展匹配逻辑</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>已关闭</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-逻辑审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>CR-002</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>OpCooperativeMatrixLengthHW缺少length检查，直接访问ops[0~2]，若SPIR-V指令长度不足3会越界</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>遗漏bounds check，其他HW指令都有length保护</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>审查HW指令的length校验一致性</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-安全性审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>CR-003</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>OpCooperativeMatrixReduceHW的reduce_mask_id和combine_op_id用get&lt;SPIRConstant&gt;强转，与layout bug(UT-017)同一模式，若mask/op为三目运算符会抛bad_cast</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>未参考layout修复模式同步修正ReduceHW的常量强转</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>审查ReduceHW实现发现与已修复的layout bug相同模式</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-一致性审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>CR-004</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>OpCooperativeMatrixReduceHW的mask只判断==0否则当Column，op只判断0/1否则当Max，未校验范围，越界值静默走错枚举</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>缺少枚举值范围校验，越界值静默处理</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>审查ReduceHW的枚举值分发逻辑</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-逻辑审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>CR-005</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>riflebird</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>OpCpAsyncTensorGlobalSharedHW未调用register_write(dst_ptr)，与StoreHW不一致，影响变量scope分析</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>OpCpAsyncTensorGlobalSharedHW未调用register_write(dst_ptr)，与StoreHW/VectorStoreHW不一致，影响变量scope分析</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>低</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>遗漏register_write调用</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>代码审查</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>审查CpAsync指令的变量追踪一致性</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>未关闭</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr"/>
-      <c r="K18" s="2" t="inlineStr"/>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>代码审查-一致性审查</t>
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>统计</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>总计 28 条</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>已关闭 24 条，未关闭 4 条</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>UT 17 条 / ST 6 条 / CR 5 条</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>高 13 / 中 11 / 低 4</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L18"/>
+  <autoFilter ref="A1:L29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Expand UT/ST summary to 39 defects
Added 11 new entries from deep code review:
- CR-006: StoreHW missing register_write(ptr)
- CR-007: VectorStoreHW missing register_write(ptr)
- CR-008: Constant expression missing SByte/UByte for CoopMatHW/CoopVecHW
- CR-009: CpAsync missing in AnalyzeVariableScopeAccessHandler
- CR-010: OpFConvert missing explicit CoopMatHW/CoopVecHW case
- ST-007: Missing LengthHW + spec constant test
- ST-008: Missing SByte/UByte component type test
- ST-009: Missing ReduceHW ternary mask/op test
- ST-010: Missing Memory Operands test for HW Load/Store
- ST-011: Missing cross-type CoopMatHW<->CoopVecHW bitcast test
- ST-012: Missing TensorMap dimensions validation test

24 closed, 15 open. UT 17 / ST 12 / CR 10. Header frozen, auto-filter.
</commit_message>
<xml_diff>
--- a/doc/hw-ut-st-summary.xlsx
+++ b/doc/hw-ut-st-summary.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="研发自测UT-ST缺陷总结表" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'研发自测UT-ST缺陷总结表'!$A$1:$L$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'研发自测UT-ST缺陷总结表'!$A$1:$L$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>OpCooperativeMatrixStoreHW操作数顺序错误：代码按(Object,Pointer)读取，实际SPIR-V定义为(Pointer,Object)，影响3处（emit、interface tracking、scope analysis）</t>
+          <t>OpCooperativeMatrixStoreHW操作数顺序错误：代码按(Object,Pointer)读取，实际为(Pointer,Object)，影响3处</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>设计规范变更时操作数顺序理解错误，未遵循标准OpStore约定（Pointer在前Object在后）</t>
+          <t>设计规范变更时操作数顺序理解错误，未遵循标准OpStore约定</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>非GLSL后端（MSL/HLSL/CPP/Reflect）对HW扩展静默生成错误代码：HW指令经default分支落入基类CompilerGLSL::emit_instruction，将GLSL intrinsic写入MSL/HLSL输出</t>
+          <t>非GLSL后端对HW扩展静默生成错误代码：HW指令经default分支落入基类emit_instruction，将GLSL intrinsic写入MSL/HLSL输出</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Vulkan GLSL输出未覆盖：所有HW shader仅有OpenGL GLSL测试，缺少--vulkan-semantics(-V)输出验证</t>
+          <t>Vulkan GLSL输出未覆盖：所有HW shader仅有OpenGL GLSL测试，缺少--vulkan-semantics输出验证</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>reject_hw_neural_extensions扩展检测用rfind("SPV_HW_",0)前缀匹配，过于宽泛，可能误拒未来其他SPV_HW_*扩展</t>
+          <t>reject_hw_neural_extensions扩展检测用rfind("SPV_HW_",0)前缀匹配，过于宽泛</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -2068,7 +2068,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>OpCooperativeMatrixReduceHW的reduce_mask_id和combine_op_id用get&lt;SPIRConstant&gt;强转，与layout bug(UT-017)同一模式，若mask/op为三目运算符会抛bad_cast</t>
+          <t>OpCooperativeMatrixReduceHW的mask/op用get&lt;SPIRConstant&gt;强转，与layout bug(UT-017)同一模式，三目运算符会抛bad_cast</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>OpCooperativeMatrixReduceHW的mask只判断==0否则当Column，op只判断0/1否则当Max，未校验范围，越界值静默走错枚举</t>
+          <t>ReduceHW的mask只判断==0否则当Column，op只判断0/1否则当Max，未校验范围，越界值静默走错枚举</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>OpCpAsyncTensorGlobalSharedHW未调用register_write(dst_ptr)，与StoreHW/VectorStoreHW不一致，影响变量scope分析</t>
+          <t>OpCpAsyncTensorGlobalSharedHW未调用register_write(dst_ptr)，影响变量scope分析</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -2217,39 +2217,633 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>CR-006</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>OpCooperativeMatrixStoreHW只调用register_write(object)，缺少register_write(ptr)，OpStore同时调用两者。写入后指向同一buffer的前转表达式不会被失效</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>与OpStore的register_write模式不一致，遗漏目标指针的写入注册</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>对比OpStore和StoreHW的register_write调用</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-一致性审查</t>
+        </is>
+      </c>
+    </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>CR-007</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>OpCooperativeVectorStoreHW同CR-006，缺少register_write(ptr)，仅调用register_write(object)</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>与OpStore的register_write模式不一致，同CR-006</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>对比OpStore和VectorStoreHW的register_write调用</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-一致性审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>CR-008</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>CoopMatHW/CoopVecHW常量表达式不支持SByte/UByte组件类型，设计规范声明s8可用但constant_expression的switch中无SByte/UByte case</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>常量表达式组件类型分支遗漏SByte/UByte，抛"Unsupported component type"</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>审查constant_expression的组件类型覆盖完整性</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-逻辑审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>CR-009</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>OpCpAsyncTensorGlobalSharedHW未在spirv_cross.cpp的AnalyzeVariableScopeAccessHandler中注册，写入共享内存的变量作用域追踪缺失</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Store类指令应在scope analysis handler中注册，CpAsync是异步store但写入目标追踪缺失</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>审查spirv_cross.cpp中HW指令的scope追踪覆盖</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-一致性审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>CR-010</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>OpFConvert未对CoopMatHW/CoopVecHW做显式处理（其他转换OpSConvert/OpUConvert/OpConvertFToS等均有），虽经type_to_glsl_constructor可工作但不一致</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>转换指令中CoopMatHW/CoopVecHW分支覆盖不完整，OpFConvert遗漏显式case</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>审查转换指令的CoopMatHW/CoopVecHW分支覆盖</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>代码审查-一致性审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>ST-007</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>缺少OpCooperativeMatrixLengthHW与spec constant维度组合的测试用例，UT-014修复后未回归验证spec constant矩阵的length()</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>测试用例未覆盖spec constant维度+LengthHW的组合场景</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>审查LengthHW测试覆盖发现spec constant维度场景缺失</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>ST-覆盖缺口</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>ST-008</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>缺少SByte/UByte组件类型的CoopMatHW/CoopVecHW测试用例，设计规范声明s8可用但测试未覆盖</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>测试用例仅覆盖Float/Half/Int/UInt/Short/UShort，遗漏8位整数</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>审查测试shader发现无int8_t/uint8_t组件类型用例</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>ST-覆盖缺口</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>ST-009</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>缺少OpCooperativeMatrixReduceHW mask/op为非常量（三目运算符）的测试用例，CR-003指出同一bad_cast模式但无回归用例</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>测试用例未覆盖mask/op为OpSelect/OpSpecConstantOp的场景</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>审查ReduceHW测试发现无常量三目运算符用例</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>ST-覆盖缺口</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>ST-010</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>缺少HW Load/Store带Memory Operands（NonPrivate/Coherent等）的测试用例，代码中忽略Memory Operands但未验证</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>测试用例未覆盖可选Memory Operands的解析路径</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>审查Load/StoreHW测试发现无Memory Operands用例</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>ST-覆盖缺口</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>ST-011</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>缺少CoopMatHW↔CoopVecHW跨类型OpBitcast测试用例，代码支持但测试仅覆盖同类型间bitcast</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>测试用例未覆盖CoopMatHW到CoopVecHW的跨类型bitcast</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>审查OpBitcast测试发现无跨类型用例</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>ST-覆盖缺口</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>ST-012</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>riflebird</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>缺少TensorMap维度参数校验测试，若SPV中dimensions=5或0，输出tensorMap5D/tensorMap0D为无效GLSL类型但未报错</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>TensorMap维度参数无范围校验，越界值静默输出无效类型名</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>代码审查</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>审查TensorMap类型发现维度无validation</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>未关闭</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>ST-覆盖缺口</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>统计</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>总计 28 条</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>已关闭 24 条，未关闭 4 条</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>UT 17 条 / ST 6 条 / CR 5 条</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>高 13 / 中 11 / 低 4</t>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>总计 39 条</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>已关闭 24 / 未关闭 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>UT 17 / ST 12 / CR 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>高 16 / 中 15 / 低 8</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L29"/>
+  <autoFilter ref="A1:L40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>